<commit_message>
alterado o nome do item na ficha da CBMM, deLUVA CUT SMART para Luva Volk Do Brasil, devido a problemas de incompatibilidade de 'CA'
</commit_message>
<xml_diff>
--- a/modelos_x_cliente/CBMM.xlsx
+++ b/modelos_x_cliente/CBMM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonardo GAP\Documents\Gerador-de-fichas-de-EPI\modelos_x_cliente\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4A8C2D-9B7F-46A3-BB80-8F96C6D36828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99490785-46C7-4255-901D-79C588549CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -183,9 +183,6 @@
     <t>CBMM ARAXÁ (MG)</t>
   </si>
   <si>
-    <t>LUVA CUT SMART</t>
-  </si>
-  <si>
     <t>Botina ANTI TORÇÃO</t>
   </si>
   <si>
@@ -199,6 +196,9 @@
   </si>
   <si>
     <t>Calça Jeans</t>
+  </si>
+  <si>
+    <t>Luva Volk Do Brasil</t>
   </si>
 </sst>
 </file>
@@ -1106,6 +1106,51 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1123,15 +1168,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1162,42 +1198,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1531,21 +1531,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:26" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="86" t="s">
+      <c r="B2" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="86"/>
-      <c r="M2" s="86"/>
-      <c r="N2" s="86"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
@@ -1560,59 +1560,59 @@
     </row>
     <row r="3" spans="2:26" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:26" s="3" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="92" t="s">
+      <c r="B4" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="96" t="s">
+      <c r="C4" s="81" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="79" t="s">
+      <c r="D4" s="91" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="90" t="s">
+      <c r="E4" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="87" t="s">
+      <c r="F4" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="88"/>
-      <c r="H4" s="89"/>
-      <c r="I4" s="73" t="s">
+      <c r="G4" s="70"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="78" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="74"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="73" t="s">
+      <c r="J4" s="79"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="78" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="74"/>
-      <c r="N4" s="75"/>
-      <c r="O4" s="70" t="s">
+      <c r="M4" s="79"/>
+      <c r="N4" s="80"/>
+      <c r="O4" s="85" t="s">
         <v>18</v>
       </c>
-      <c r="P4" s="71"/>
-      <c r="Q4" s="72"/>
-      <c r="R4" s="73" t="s">
+      <c r="P4" s="86"/>
+      <c r="Q4" s="87"/>
+      <c r="R4" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="S4" s="74"/>
-      <c r="T4" s="75"/>
-      <c r="U4" s="76" t="s">
+      <c r="S4" s="79"/>
+      <c r="T4" s="80"/>
+      <c r="U4" s="88" t="s">
         <v>26</v>
       </c>
-      <c r="V4" s="74"/>
-      <c r="W4" s="75"/>
-      <c r="X4" s="76" t="s">
+      <c r="V4" s="79"/>
+      <c r="W4" s="80"/>
+      <c r="X4" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="Y4" s="74"/>
-      <c r="Z4" s="75"/>
+      <c r="Y4" s="79"/>
+      <c r="Z4" s="80"/>
     </row>
     <row r="5" spans="2:26" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="93"/>
-      <c r="C5" s="97"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="91"/>
+      <c r="B5" s="75"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="73"/>
       <c r="F5" s="8" t="s">
         <v>20</v>
       </c>
@@ -1676,17 +1676,17 @@
       </c>
     </row>
     <row r="6" spans="2:26" ht="25.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="94">
+      <c r="B6" s="76">
         <v>3</v>
       </c>
       <c r="C6" s="35">
         <v>3</v>
       </c>
       <c r="D6" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E6" s="67" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F6" s="14"/>
       <c r="G6" s="27"/>
@@ -1711,12 +1711,12 @@
       <c r="Z6" s="16"/>
     </row>
     <row r="7" spans="2:26" ht="25.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="95"/>
+      <c r="B7" s="77"/>
       <c r="C7" s="37">
         <v>1</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E7" s="66" t="s">
         <v>40</v>
@@ -1744,12 +1744,12 @@
       <c r="Z7" s="22"/>
     </row>
     <row r="8" spans="2:26" ht="25.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="95"/>
+      <c r="B8" s="77"/>
       <c r="C8" s="37">
         <v>1</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E8" s="40" t="s">
         <v>32</v>
@@ -1777,7 +1777,7 @@
       <c r="Z8" s="22"/>
     </row>
     <row r="9" spans="2:26" ht="25.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="95"/>
+      <c r="B9" s="77"/>
       <c r="C9" s="37">
         <v>2</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>50</v>
       </c>
       <c r="E9" s="48" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F9" s="20"/>
       <c r="G9" s="4"/>
@@ -1810,7 +1810,7 @@
       <c r="Z9" s="22"/>
     </row>
     <row r="10" spans="2:26" ht="25.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="95"/>
+      <c r="B10" s="77"/>
       <c r="C10" s="39">
         <v>1</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>43</v>
       </c>
       <c r="E10" s="49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F10" s="28"/>
       <c r="G10" s="26"/>
@@ -1936,7 +1936,7 @@
       <c r="Z13" s="30"/>
     </row>
     <row r="14" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="77" t="s">
+      <c r="B14" s="89" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="59">
@@ -1969,7 +1969,7 @@
       <c r="Z14" s="22"/>
     </row>
     <row r="15" spans="2:26" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="78"/>
+      <c r="B15" s="90"/>
       <c r="C15" s="62">
         <v>1</v>
       </c>
@@ -2000,13 +2000,13 @@
       <c r="Z15" s="7"/>
     </row>
     <row r="16" spans="2:26" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="78"/>
+      <c r="B16" s="90"/>
       <c r="C16" s="62">
         <v>1</v>
       </c>
       <c r="D16" s="63"/>
       <c r="E16" s="52" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F16" s="20"/>
       <c r="G16" s="4"/>
@@ -2031,7 +2031,7 @@
       <c r="Z16" s="7"/>
     </row>
     <row r="17" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="78"/>
+      <c r="B17" s="90"/>
       <c r="C17" s="62">
         <v>1</v>
       </c>
@@ -2062,7 +2062,7 @@
       <c r="Z17" s="22"/>
     </row>
     <row r="18" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="78"/>
+      <c r="B18" s="90"/>
       <c r="C18" s="62">
         <v>1</v>
       </c>
@@ -2093,7 +2093,7 @@
       <c r="Z18" s="22"/>
     </row>
     <row r="19" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="78"/>
+      <c r="B19" s="90"/>
       <c r="C19" s="62">
         <v>1</v>
       </c>
@@ -2125,11 +2125,11 @@
     </row>
     <row r="20" spans="2:26" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="42"/>
-      <c r="C20" s="81" t="s">
+      <c r="C20" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="82"/>
-      <c r="E20" s="83"/>
+      <c r="D20" s="94"/>
+      <c r="E20" s="95"/>
       <c r="F20" s="32"/>
       <c r="G20" s="41" t="s">
         <v>37</v>
@@ -2141,11 +2141,11 @@
     </row>
     <row r="21" spans="2:26" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="42"/>
-      <c r="C21" s="81" t="s">
+      <c r="C21" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="82"/>
-      <c r="E21" s="83"/>
+      <c r="D21" s="94"/>
+      <c r="E21" s="95"/>
       <c r="F21" s="32"/>
       <c r="G21" s="41" t="s">
         <v>37</v>
@@ -2157,11 +2157,11 @@
     </row>
     <row r="22" spans="2:26" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="42"/>
-      <c r="C22" s="81" t="s">
+      <c r="C22" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="82"/>
-      <c r="E22" s="83"/>
+      <c r="D22" s="94"/>
+      <c r="E22" s="95"/>
       <c r="G22" s="41" t="s">
         <v>36</v>
       </c>
@@ -2172,10 +2172,10 @@
     </row>
     <row r="23" spans="2:26" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="42"/>
-      <c r="C23" s="84" t="s">
+      <c r="C23" s="96" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="84"/>
+      <c r="D23" s="96"/>
       <c r="E23" s="54" t="s">
         <v>47</v>
       </c>
@@ -2186,16 +2186,16 @@
       <c r="Z23" s="44"/>
     </row>
     <row r="24" spans="2:26" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="68" t="s">
+      <c r="B24" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="69"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="85" t="s">
-        <v>51</v>
-      </c>
-      <c r="F24" s="85"/>
-      <c r="G24" s="85"/>
+      <c r="C24" s="84"/>
+      <c r="D24" s="84"/>
+      <c r="E24" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" s="97"/>
+      <c r="G24" s="97"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
       <c r="J24" s="33"/>
@@ -2227,14 +2227,6 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0"/>
   <mergeCells count="20">
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="L4:N4"/>
-    <mergeCell ref="C4:C5"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="O4:Q4"/>
     <mergeCell ref="R4:T4"/>
@@ -2247,6 +2239,14 @@
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="E24:G24"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="C4:C5"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2255,15 +2255,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="3a415345-6a39-4751-b960-4fc8f12baef7">
@@ -2273,6 +2264,15 @@
     <MediaLengthInSeconds xmlns="3a415345-6a39-4751-b960-4fc8f12baef7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2517,20 +2517,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A9F4E51-4DE3-4214-9644-9D529D38719F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6192A4F-43EB-47CE-AABA-403827665463}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="3a415345-6a39-4751-b960-4fc8f12baef7"/>
     <ds:schemaRef ds:uri="74ad866f-79dd-4f7a-ba3c-81e3e663768c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A9F4E51-4DE3-4214-9644-9D529D38719F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>